<commit_message>
updated submission to use .env
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729E5C0E-8EF1-4CE4-9815-5CD84A2D140A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234225A6-413A-4854-84AB-522438F42367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
last best leaderboard score
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF552087-7732-4E1D-8214-370B661EC849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA5A13C-1CE0-43F8-A0FC-9D269BE4682A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Exp#</t>
   </si>
@@ -52,6 +52,18 @@
   </si>
   <si>
     <t>ResNet34</t>
+  </si>
+  <si>
+    <t>pgd_resnet34_eps6_adv05</t>
+  </si>
+  <si>
+    <t>pgd_resnet34_eps8_adv05</t>
+  </si>
+  <si>
+    <t>Not improved</t>
+  </si>
+  <si>
+    <t>pgd_resnet34_eps6_steps7_adv05</t>
   </si>
 </sst>
 </file>
@@ -389,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -440,7 +452,50 @@
         <v>0.46563199999999999</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.46590799999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0.48163099999999998</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
params column added updated
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA5A13C-1CE0-43F8-A0FC-9D269BE4682A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE2D1D2F-E7C2-46E6-9B4D-B12CBB6615F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>Exp#</t>
   </si>
@@ -64,6 +64,30 @@
   </si>
   <si>
     <t>pgd_resnet34_eps6_steps7_adv05</t>
+  </si>
+  <si>
+    <t>python train_pgd.py `
+  --npz_path ./data/train.npz `
+  --output_dir runs/pgd_resnet34_eps6_steps7_adv05_long `
+  --model_name resnet34 `
+  --epochs 120 `
+  --batch_size 128 `
+  --val_size 0.1 `
+  --lr 0.05 `
+  --weight_decay 5e-4 `
+  --train_eps 0.023529412 `
+  --train_alpha 0.003921568 `
+  --train_steps 7 `
+  --adv_weight 0.5 `
+  --eval_eps 0.031372549 `
+  --eval_alpha 0.007843137 `
+  --eval_steps 20 `
+  --patience 25 `
+  --min_epochs 40 `
+  --clean_acc_floor 0.56</t>
+  </si>
+  <si>
+    <t>Params</t>
   </si>
 </sst>
 </file>
@@ -113,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -121,6 +145,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,16 +426,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
     <col min="3" max="3" width="44.5703125" style="2" customWidth="1"/>
     <col min="4" max="4" width="103.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="94.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -423,8 +449,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -438,7 +467,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -452,7 +481,7 @@
         <v>0.46563199999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -466,7 +495,7 @@
         <v>0.46590799999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -480,7 +509,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -492,6 +521,9 @@
       </c>
       <c r="D6" s="2">
         <v>0.48163099999999998</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
best score with resnet50
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE2D1D2F-E7C2-46E6-9B4D-B12CBB6615F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49A39AF-9D8E-437E-9036-39039CE2CAB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
   <si>
     <t>Exp#</t>
   </si>
@@ -88,6 +89,15 @@
   </si>
   <si>
     <t>Params</t>
+  </si>
+  <si>
+    <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv05_long --model_name resnet50 --epochs 120 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.5 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
+  </si>
+  <si>
+    <t>ResNet50</t>
+  </si>
+  <si>
+    <t>pgd_resnet50_eps6_steps7_adv05</t>
   </si>
 </sst>
 </file>
@@ -145,7 +155,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -509,7 +521,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -524,10 +536,67 @@
       </c>
       <c r="E6" s="3" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0.54373099999999996</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C595A2-272A-4798-A105-A83B5DFCCF60}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="16" style="2" customWidth="1"/>
+    <col min="3" max="3" width="44.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="94.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>164882</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated best with adv_weight 0.6 and resnet50
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49A39AF-9D8E-437E-9036-39039CE2CAB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DE4EF3-D674-41C5-A198-223D29D3587E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,17 +16,26 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
   <si>
     <t>Exp#</t>
   </si>
@@ -98,6 +107,15 @@
   </si>
   <si>
     <t>pgd_resnet50_eps6_steps7_adv05</t>
+  </si>
+  <si>
+    <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv06_long --model_name resnet50 --epochs 120 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.6 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
+  </si>
+  <si>
+    <t>Cluster Run ID</t>
+  </si>
+  <si>
+    <t>pgd_resnet50_eps6_steps7_adv06</t>
   </si>
 </sst>
 </file>
@@ -147,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -157,6 +175,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -438,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -446,9 +467,10 @@
     <col min="3" max="3" width="44.5703125" style="2" customWidth="1"/>
     <col min="4" max="4" width="103.42578125" style="2" customWidth="1"/>
     <col min="5" max="5" width="94.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -464,8 +486,11 @@
       <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -479,7 +504,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -493,7 +518,7 @@
         <v>0.46563199999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -507,7 +532,7 @@
         <v>0.46590799999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -521,7 +546,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -538,7 +563,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -554,16 +579,39 @@
       <c r="E7" t="s">
         <v>15</v>
       </c>
+      <c r="F7">
+        <v>164882</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0.55972999999999995</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8">
+        <v>165012</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C595A2-272A-4798-A105-A83B5DFCCF60}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -573,7 +621,7 @@
     <col min="5" max="5" width="94.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -590,10 +638,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F2">
-        <v>164882</v>
-      </c>
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed excel merge conflict
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7580439-F364-48D3-AD1B-5D432C21EC02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D30C43C8-869E-4092-9D4A-B8DC385D25F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Exp#</t>
   </si>
@@ -607,149 +607,10 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C595A2-272A-4798-A105-A83B5DFCCF60}">
-  <dimension ref="A1:F8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BACED8CC-D10B-4971-B2C1-F924C98E4EE2}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="2" width="16" style="2" customWidth="1"/>
-    <col min="3" max="3" width="44.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="42.7109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="94.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.46563199999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.46590799999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="285" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0.48163099999999998</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0.54373099999999996</v>
-      </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7">
-        <v>164882</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0.55972999999999995</v>
-      </c>
-      <c r="E8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8">
-        <v>165012</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated sheet for resnet50 experiment
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F5FB61-601F-4463-A27D-151649C1D6B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFE48AB-E7FA-4C1E-8C58-0780840F4FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
   <si>
     <t>Exp#</t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>pgd_resnet50_eps6_steps10_adv05_btch64</t>
+  </si>
+  <si>
+    <t>pgd_resnet50_eps6_steps7_adv045</t>
+  </si>
+  <si>
+    <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv045_long --model_name resnet50 --epochs 120 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.45 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
   </si>
 </sst>
 </file>
@@ -459,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -615,6 +621,26 @@
       </c>
       <c r="D9" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10">
+        <v>165068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
best with 150 epochs
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E4E2C70-8C32-451E-A939-7E681F3D6CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07AFC4EE-49AB-43FB-A0B8-73B0B990588D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
   <si>
     <t>Exp#</t>
   </si>
@@ -125,6 +125,12 @@
   </si>
   <si>
     <t>pgd_resnet50_eps6_steps7_adv07</t>
+  </si>
+  <si>
+    <t>pgd_resnet50_eps6_steps7_adv06_epochs150</t>
+  </si>
+  <si>
+    <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv06_epochs150 --model_name resnet50 --epochs 150 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.6 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
   </si>
 </sst>
 </file>
@@ -174,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -182,7 +188,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -563,7 +568,7 @@
       <c r="D6" s="2">
         <v>0.48163099999999998</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -647,6 +652,26 @@
       </c>
       <c r="D11" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.56553699999999996</v>
+      </c>
+      <c r="E12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12">
+        <v>165167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
best with resnet50 ema
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14AC4BC9-355E-4CD1-AD94-1149C602D950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{045782E5-5B70-419C-8E42-27946D48C918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="31">
   <si>
     <t>Exp#</t>
   </si>
@@ -140,6 +140,12 @@
   </si>
   <si>
     <t>pgd_resnet34_eps6_steps7_adv06_ema</t>
+  </si>
+  <si>
+    <t>pgd_resnet50_eps6_steps7_adv06_ema</t>
+  </si>
+  <si>
+    <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd_ema.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv06_ema --model_name resnet50 --epochs 150 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.6 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56 --use_ema --ema_decay 0.999</t>
   </si>
 </sst>
 </file>
@@ -477,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -723,6 +729,26 @@
       </c>
       <c r="D15" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.57162000000000002</v>
+      </c>
+      <c r="E16" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16">
+        <v>165552</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correction in experiment file
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Robustness\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{045782E5-5B70-419C-8E42-27946D48C918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4ED8005-1B5C-482E-AC4B-4F08BE72E4DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -722,7 +722,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
best with seed 24, 150 epochs
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB401A8-94DB-4AEB-AE5F-A917658F41DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BF81F8-8D0A-4236-8988-C8E7E4FE329E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
   <si>
     <t>Exp#</t>
   </si>
@@ -179,6 +179,12 @@
   </si>
   <si>
     <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv06_epochs150_seed12 --model_name resnet50 --epochs 150 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --seed 12 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.6 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
+  </si>
+  <si>
+    <t>pgd_resnet50_eps6_steps7_adv06_epochs150_seed24</t>
+  </si>
+  <si>
+    <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv06_epochs150_seed24 --model_name resnet50 --epochs 150 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --seed 24 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.6 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
   </si>
 </sst>
 </file>
@@ -516,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -910,6 +916,26 @@
       </c>
       <c r="F23">
         <v>165952</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="2">
+        <v>0.57821800000000001</v>
+      </c>
+      <c r="E24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F24">
+        <v>166004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
best with seed 20, epochs 200
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 3\tml2026-team_XLIII-assignment_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BF81F8-8D0A-4236-8988-C8E7E4FE329E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CA65FC7-1328-42FE-9ACE-6CCF26D84266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="46">
   <si>
     <t>Exp#</t>
   </si>
@@ -185,6 +185,12 @@
   </si>
   <si>
     <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv06_epochs150_seed24 --model_name resnet50 --epochs 150 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --seed 24 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.6 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
+  </si>
+  <si>
+    <t>pgd_resnet50_eps6_steps7_adv06_epochs200_seed20</t>
+  </si>
+  <si>
+    <t>/home/atml_team040/tml2026-team_XLIII-assignment_3/train_pgd.py --npz_path /home/atml_team040/tml2026-team_XLIII-assignment_3/train.npz --output_dir /home/atml_team040/tml2026-team_XLIII-assignment_3/runs/pgd_resnet50_eps6_steps7_adv06_epochs200_seed20 --model_name resnet50 --epochs 200 --batch_size 128 --val_size 0.1 --lr 0.05 --weight_decay 5e-4 --seed 20 --train_eps 0.023529412 --train_alpha 0.003921568 --train_steps 7 --adv_weight 0.6 --eval_eps 0.031372549 --eval_alpha 0.007843137 --eval_steps 20 --patience 25 --min_epochs 40 --clean_acc_floor 0.56</t>
   </si>
 </sst>
 </file>
@@ -522,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -936,6 +942,26 @@
       </c>
       <c r="F24">
         <v>166004</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.58730300000000002</v>
+      </c>
+      <c r="E25" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25">
+        <v>166005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>